<commit_message>
Add conditional Cloudflare free tier to intake cost estimate
</commit_message>
<xml_diff>
--- a/INTAKE_COST_ESTIMATE.xlsx
+++ b/INTAKE_COST_ESTIMATE.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Inputs" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Evidence and prices" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Cloudflare candidate" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Inputs!$A$3:$E$35</definedName>
@@ -103,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="209">
   <si>
     <t xml:space="preserve">ArabicaAI | Intake cost sensitivity</t>
   </si>
@@ -156,6 +157,12 @@
     <t xml:space="preserve">Change pale-yellow values on Inputs. Blue-green cells on Scenarios recalculate in Excel/LibreOffice.</t>
   </si>
   <si>
+    <t xml:space="preserve">Cloudflare candidate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worker + D1 may have $0 fixed cloud cost inside Free limits; a code migration and CPU/D1 checks are required. See its separate sheet.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not in estimate</t>
   </si>
   <si>
@@ -165,7 +172,7 @@
     <t xml:space="preserve">Reviewed</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-28; prices should be rechecked before spending. No credits assumed.</t>
+    <t xml:space="preserve">2026-09-29; prices should be rechecked before spending. No credits assumed.</t>
   </si>
   <si>
     <t xml:space="preserve">Editable inputs | yellow = change with evidence</t>
@@ -655,19 +662,89 @@
   </si>
   <si>
     <t xml:space="preserve">This workbook is not a calculator export</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloudflare Workers Free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100,000 requests/day, 10 ms CPU/request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://developers.cloudflare.com/workers/platform/pricing/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditional free candidate; this report has no measured CPU usage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloudflare D1 Free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5M rows read/day, 100k rows written/day, 500 MB per database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://developers.cloudflare.com/d1/platform/limits/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No measured D1 row scans or storage forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloudflare Worker + D1 | conditional Free plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A connected GitHub repo does not migrate the current PostgreSQL demo. The Worker variant must pass live CPU and D1 checks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planned Worker req/day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free req/day cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request headroom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request-cap check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Illustrative AI USD/month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potential fixed hosting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$0 only while Worker and D1 stay inside Free quotas; not a capacity promise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still unmeasured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPU ms/request (Free: 10 ms); D1 rows read/write, DB size, retries, static requests, peak traffic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model charges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI usage in column G is hypothetical and billed separately from Cloudflare. Current demo uses no model.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Readiness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 9,000/day scenario has only 10,000 requests/day headroom under the assumed 10 calls/episode.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.00"/>
     <numFmt numFmtId="168" formatCode="\$#,##0.00;[RED]&quot;($&quot;#,##0.00\)"/>
     <numFmt numFmtId="169" formatCode="\$#,##0.0000;[RED]&quot;($&quot;#,##0.0000\)"/>
+    <numFmt numFmtId="170" formatCode="General"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -824,7 +901,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -883,6 +960,18 @@
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1354,11 +1443,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="2224126"/>
-        <c:axId val="93463012"/>
+        <c:axId val="10581119"/>
+        <c:axId val="59633388"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2224126"/>
+        <c:axId val="10581119"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1424,7 +1513,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93463012"/>
+        <c:crossAx val="59633388"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1432,7 +1521,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93463012"/>
+        <c:axId val="59633388"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1508,7 +1597,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2224126"/>
+        <c:crossAx val="10581119"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1862,15 +1951,20 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2"/>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1878,10 +1972,10 @@
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1915,7 +2009,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1924,538 +2018,538 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>4118</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>365</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>30</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>10</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>0.1</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>12000</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>2000</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B16" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D16" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B17" s="7" t="n">
         <v>7</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="7" t="n">
         <v>6</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>0.3</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>24</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>20</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>0.05</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B24" s="7" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>30</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B28" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D28" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B29" s="7" t="n">
         <v>0</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D31" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>102</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B35" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2492,7 +2586,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2515,7 +2609,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2538,66 +2632,66 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">Inputs!B5/Inputs!B6*Inputs!B35</f>
@@ -2674,7 +2768,7 @@
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B6" s="9" t="n">
         <v>100</v>
@@ -2750,7 +2844,7 @@
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>900</v>
@@ -2826,7 +2920,7 @@
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>9000</v>
@@ -2902,10 +2996,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -2927,10 +3021,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -2952,10 +3046,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -3000,7 +3094,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -3011,7 +3105,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3019,13 +3113,13 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>9</v>
@@ -3033,114 +3127,142 @@
     </row>
     <row r="4" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -3153,6 +3275,8 @@
     <hyperlink ref="C9" r:id="rId3" display="https://render.com/pricing"/>
     <hyperlink ref="C10" r:id="rId4" display="https://aws.amazon.com/free/"/>
     <hyperlink ref="C11" r:id="rId5" display="https://calculator.aws/"/>
+    <hyperlink ref="C12" r:id="rId6" display="https://developers.cloudflare.com/workers/platform/pricing/"/>
+    <hyperlink ref="C13" r:id="rId7" display="https://developers.cloudflare.com/d1/platform/limits/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3162,4 +3286,253 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="31"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="str">
+        <f aca="false">Scenarios!A5</f>
+        <v>2025 V1 complaint proxy</v>
+      </c>
+      <c r="B5" s="15" t="n">
+        <f aca="false">Scenarios!B5</f>
+        <v>11.2821917808219</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <f aca="false">B5*Inputs!B9</f>
+        <v>112.821917808219</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <f aca="false">D5-C5</f>
+        <v>99887.1780821918</v>
+      </c>
+      <c r="F5" s="0" t="str">
+        <f aca="false">IF(C5&lt;=D5,"under request cap","over request cap")</f>
+        <v>under request cap</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <f aca="false">Scenarios!J5</f>
+        <v>1.62463561643836</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="str">
+        <f aca="false">Scenarios!A6</f>
+        <v>100/day test</v>
+      </c>
+      <c r="B6" s="15" t="n">
+        <f aca="false">Scenarios!B6</f>
+        <v>100</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <f aca="false">B6*Inputs!B9</f>
+        <v>1000</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <f aca="false">D6-C6</f>
+        <v>99000</v>
+      </c>
+      <c r="F6" s="0" t="str">
+        <f aca="false">IF(C6&lt;=D6,"under request cap","over request cap")</f>
+        <v>under request cap</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <f aca="false">Scenarios!J6</f>
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="str">
+        <f aca="false">Scenarios!A7</f>
+        <v>900/day all-contact stress</v>
+      </c>
+      <c r="B7" s="15" t="n">
+        <f aca="false">Scenarios!B7</f>
+        <v>900</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <f aca="false">B7*Inputs!B9</f>
+        <v>9000</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <f aca="false">D7-C7</f>
+        <v>91000</v>
+      </c>
+      <c r="F7" s="0" t="str">
+        <f aca="false">IF(C7&lt;=D7,"under request cap","over request cap")</f>
+        <v>under request cap</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <f aca="false">Scenarios!J7</f>
+        <v>129.6</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="str">
+        <f aca="false">Scenarios!A8</f>
+        <v>9,000/day stress</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <f aca="false">Scenarios!B8</f>
+        <v>9000</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <f aca="false">B8*Inputs!B9</f>
+        <v>90000</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <f aca="false">D8-C8</f>
+        <v>10000</v>
+      </c>
+      <c r="F8" s="0" t="str">
+        <f aca="false">IF(C8&lt;=D8,"under request cap","over request cap")</f>
+        <v>under request cap</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <f aca="false">Scenarios!J8</f>
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>